<commit_message>
Fix Python environment selection on macOS
</commit_message>
<xml_diff>
--- a/题库/PY选择题.xlsx
+++ b/题库/PY选择题.xlsx
@@ -864,12 +864,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FF0F1115"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
       <t>给出如下代码</t>
     </r>
     <r>
@@ -1657,7 +1651,7 @@
         <rFont val="Segoe UI"/>
         <charset val="134"/>
       </rPr>
-      <t>”)</t>
+      <t>”))</t>
     </r>
   </si>
   <si>
@@ -1790,12 +1784,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FF0F1115"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
       <t>下列程序的输出结果是（</t>
     </r>
     <r>
@@ -1829,7 +1817,7 @@
 f.seek(0) 
 c=f.read(2) 
 print(c) 
-f.close0</t>
+f.close()</t>
     </r>
   </si>
   <si>

</xml_diff>